<commit_message>
google sheet preprod version
</commit_message>
<xml_diff>
--- a/dane_obozu.xlsx
+++ b/dane_obozu.xlsx
@@ -12,6 +12,12 @@
     <sheet name="schedule" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="events" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="personal_plans" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Grupa" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Americano" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Turniej tie breakowy" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Turniej singlowy" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Wycieczki" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Grupa_wyjatki" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,6 +516,146 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>participant_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>day_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Anna Kowalska</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Celina Wiśniewska</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>day_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>participants</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>trainer</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>court</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>training_time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Grupa 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Anna Kowalska, Celina Wiśniewska</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Trener Paweł</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Kort 5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -828,16 +974,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -858,22 +1002,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>court</t>
+          <t>event_labels</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>with_players</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>with_coach</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>event_labels</t>
+          <t>note</t>
         </is>
       </c>
     </row>
@@ -890,25 +1024,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kort 1</t>
+          <t>Wycieczka do Side</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bartek Nowak</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Trener Tomek</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Zbiórka przy recepcji</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -918,39 +1046,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kort 2</t>
+          <t>Wieczór integracyjny</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Celina Wiśniewska</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Trenerka Natalia</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Trening z trenerem</t>
+          <t>Strój sportowy</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Anna Kowalska</t>
+          <t>Bartek Nowak</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -960,122 +1078,328 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Kort 3</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Bartek Nowak</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Turniej – Grupa A</t>
-        </is>
-      </c>
+          <t>Wieczór integracyjny</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Celina Wiśniewska</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sesja fizjo</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gabinet 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>participant_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>trainer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>court</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>training_time</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>day_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Anna Kowalska</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Grupa 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Trener Tomek</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Kort 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Bartek Nowak</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Grupa 1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Trener Tomek</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Kort 1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Celina Wiśniewska</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Grupa 2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Trenerka Natalia</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Kort 2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Kort 1</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>participant_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>day_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Anna Kowalska</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Bartek Nowak</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Kort 4</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Trener Tomek</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Trening z trenerem</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>participant_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>day_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Celina Wiśniewska</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Kort 2</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>participant_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>day_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Anna Kowalska</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Trener Paweł</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Trening z trenerem</t>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bartek Nowak</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>

</xml_diff>